<commit_message>
Updated output files: refined plots with extracted slopes, derivative magnitudes, and corrected Horner analysis
</commit_message>
<xml_diff>
--- a/output/analysis_results.xlsx
+++ b/output/analysis_results.xlsx
@@ -465,211 +465,211 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>1e-06</v>
       </c>
       <c r="B2" t="n">
         <v>2950.5</v>
       </c>
       <c r="C2" t="n">
-        <v>1001</v>
+        <v>1000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1.5</v>
+        <v>0.500001</v>
       </c>
       <c r="B3" t="n">
         <v>2945.3</v>
       </c>
       <c r="C3" t="n">
-        <v>667.6666666666666</v>
+        <v>2000.996000008</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>1.000001</v>
       </c>
       <c r="B4" t="n">
         <v>2940.8</v>
       </c>
       <c r="C4" t="n">
-        <v>501</v>
+        <v>1000.999000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3</v>
+        <v>2.000001</v>
       </c>
       <c r="B5" t="n">
         <v>2932.1</v>
       </c>
       <c r="C5" t="n">
-        <v>334.3333333333333</v>
+        <v>500.9997500001249</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>4.000001</v>
       </c>
       <c r="B6" t="n">
         <v>2920.5</v>
       </c>
       <c r="C6" t="n">
-        <v>201</v>
+        <v>250.9999375000156</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>7.5</v>
+        <v>6.500001</v>
       </c>
       <c r="B7" t="n">
         <v>2910.2</v>
       </c>
       <c r="C7" t="n">
-        <v>134.3333333333333</v>
+        <v>154.8461301775184</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>10</v>
+        <v>9.000000999999999</v>
       </c>
       <c r="B8" t="n">
         <v>2902.8</v>
       </c>
       <c r="C8" t="n">
-        <v>101</v>
+        <v>112.1110987654335</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>15</v>
+        <v>14.000001</v>
       </c>
       <c r="B9" t="n">
         <v>2890.3</v>
       </c>
       <c r="C9" t="n">
-        <v>67.66666666666667</v>
+        <v>72.42856632653098</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>20</v>
+        <v>19.000001</v>
       </c>
       <c r="B10" t="n">
         <v>2880.5</v>
       </c>
       <c r="C10" t="n">
-        <v>51</v>
+        <v>53.63157617728546</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>30</v>
+        <v>29.000001</v>
       </c>
       <c r="B11" t="n">
         <v>2865.2</v>
       </c>
       <c r="C11" t="n">
-        <v>34.33333333333334</v>
+        <v>35.48275743162905</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>50</v>
+        <v>49.000001</v>
       </c>
       <c r="B12" t="n">
         <v>2845.1</v>
       </c>
       <c r="C12" t="n">
-        <v>21</v>
+        <v>21.408162848813</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>75</v>
+        <v>74.000001</v>
       </c>
       <c r="B13" t="n">
         <v>2825</v>
       </c>
       <c r="C13" t="n">
-        <v>14.33333333333333</v>
+        <v>14.51351333089847</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>100</v>
+        <v>99.000001</v>
       </c>
       <c r="B14" t="n">
         <v>2810.3</v>
       </c>
       <c r="C14" t="n">
-        <v>11</v>
+        <v>11.1010099989797</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>150</v>
+        <v>149.000001</v>
       </c>
       <c r="B15" t="n">
         <v>2790.5</v>
       </c>
       <c r="C15" t="n">
-        <v>7.666666666666667</v>
+        <v>7.711409350930138</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>200</v>
+        <v>199.000001</v>
       </c>
       <c r="B16" t="n">
         <v>2775.2</v>
       </c>
       <c r="C16" t="n">
-        <v>6</v>
+        <v>6.025125602888815</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>300</v>
+        <v>299.000001</v>
       </c>
       <c r="B17" t="n">
         <v>2750.8</v>
       </c>
       <c r="C17" t="n">
-        <v>4.333333333333333</v>
+        <v>4.344481594165613</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>500</v>
+        <v>499.000001</v>
       </c>
       <c r="B18" t="n">
         <v>2720.3</v>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>3.004008012016016</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>750</v>
+        <v>749.000001</v>
       </c>
       <c r="B19" t="n">
         <v>2695.1</v>
       </c>
       <c r="C19" t="n">
-        <v>2.333333333333333</v>
+        <v>2.335113482863667</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1000</v>
+        <v>999.000001</v>
       </c>
       <c r="B20" t="n">
         <v>2675.5</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>2.001000999998998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>